<commit_message>
Added Welsh validtion check for Germany
</commit_message>
<xml_diff>
--- a/src/test/resources/welsh-data.xlsx
+++ b/src/test/resources/welsh-data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\johnwhitfield\workspace\euvat-ui-tests\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F514306-168E-4030-889B-AF28F7D00FA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E944EF58-26D1-4DDA-9F59-42651EE0D8A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="16663" windowHeight="9772" firstSheet="17" activeTab="22" xr2:uid="{397487DB-51A4-426B-A59F-CD3C6328FFCE}"/>
+    <workbookView xWindow="-16560" yWindow="-16320" windowWidth="29040" windowHeight="15720" firstSheet="17" activeTab="23" xr2:uid="{397487DB-51A4-426B-A59F-CD3C6328FFCE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet11" sheetId="11" r:id="rId1"/>
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1755" uniqueCount="722">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1728" uniqueCount="717">
   <si>
     <t xml:space="preserve">English </t>
   </si>
@@ -2111,21 +2111,9 @@
     <t>Dewiswch ‘Iawn’ os ydych am dynnu’r trydydd cod SIC</t>
   </si>
   <si>
-    <t>https://eu-vat-prototype-3c83fc449f97.herokuapp.com/sprint-11/supplier-tax-numbers-simp-invoice</t>
-  </si>
-  <si>
-    <t>https://confluence.tools.tax.service.gov.uk/spaces/RBD/pages/1314619446/RA8.1.1+-+Select+the+supplier+tax+numbers+shown+on+the+invoice</t>
-  </si>
-  <si>
-    <t>Dewiswch rifau treth y cyflenwyr a ddangosir ar yr anfoneb - TAW yr UE - GOV.UK </t>
-  </si>
-  <si>
     <t>Dewiswch rifau treth y cyflenwyr a ddangosir ar yr anfoneb</t>
   </si>
   <si>
-    <t>supplierTaxNumber.caption</t>
-  </si>
-  <si>
     <t>supplierTaxNumber.title</t>
   </si>
   <si>
@@ -2165,15 +2153,6 @@
     <t>Nid oes gennyf unrhyw un o’r rhain ar yr anfoneb</t>
   </si>
   <si>
-    <t>https://eu-vat-prototype-3c83fc449f97.herokuapp.com/sprint-11/supplier-tax-identifier</t>
-  </si>
-  <si>
-    <t>https://confluence.tools.tax.service.gov.uk/spaces/RBD/pages/1314619458/RA8.1.2+-+What+is+the+supplier%E2%80%99s+tax+identifier+number</t>
-  </si>
-  <si>
-    <t>Beth yw rhif dynodi treth y cyflenwr? - TAW yr UE - GOV.UK </t>
-  </si>
-  <si>
     <t>Beth yw rhif dynodi treth y cyflenwr?</t>
   </si>
   <si>
@@ -2226,6 +2205,12 @@
   </si>
   <si>
     <t>/supplier-tax-identifier-number</t>
+  </si>
+  <si>
+    <t>Beth yw rhif dynodi treth y cyflenwr? - TAW yr UE - GOV.UK</t>
+  </si>
+  <si>
+    <t>Dewiswch rifau treth y cyflenwyr a ddangosir ar yr anfoneb - TAW yr UE - GOV.UK</t>
   </si>
 </sst>
 </file>
@@ -3114,148 +3099,6 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing20.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>349704</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>95241</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>17</xdr:col>
-      <xdr:colOff>58376</xdr:colOff>
-      <xdr:row>31</xdr:row>
-      <xdr:rowOff>105696</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Picture 2">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{479A06ED-BE68-C9E8-4E33-AA732CE6FC92}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="14418129" y="1095366"/>
-          <a:ext cx="6480947" cy="4865483"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>33</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>19</xdr:col>
-      <xdr:colOff>344077</xdr:colOff>
-      <xdr:row>65</xdr:row>
-      <xdr:rowOff>38914</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Picture 3">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{601C4208-B56C-23E1-1E62-242ACD5D40C4}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="14068425" y="6219825"/>
-          <a:ext cx="8430802" cy="5830114"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing21.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>19</xdr:col>
-      <xdr:colOff>591761</xdr:colOff>
-      <xdr:row>36</xdr:row>
-      <xdr:rowOff>115009</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Picture 3">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{574E30C6-B520-7CAF-B96B-6041CAAA7F7C}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="14068425" y="1800225"/>
-          <a:ext cx="8678486" cy="5077534"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
 <file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
@@ -9411,7 +9254,7 @@
         <v>25</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>716</v>
+        <v>709</v>
       </c>
       <c r="E4" s="3"/>
       <c r="F4" s="3"/>
@@ -9437,7 +9280,7 @@
         <v>17</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>718</v>
+        <v>711</v>
       </c>
       <c r="E5" s="3"/>
       <c r="F5" s="3"/>
@@ -9515,7 +9358,7 @@
         <v>25</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>716</v>
+        <v>709</v>
       </c>
       <c r="E8" s="3"/>
       <c r="F8" s="3"/>
@@ -15502,7 +15345,7 @@
         <v>25</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>716</v>
+        <v>709</v>
       </c>
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>
@@ -15517,7 +15360,7 @@
         <v>17</v>
       </c>
       <c r="C2" s="18" t="s">
-        <v>717</v>
+        <v>710</v>
       </c>
       <c r="D2" s="3"/>
       <c r="E2" s="3"/>
@@ -15562,7 +15405,7 @@
         <v>25</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>716</v>
+        <v>709</v>
       </c>
       <c r="D5" s="3"/>
       <c r="E5" s="3"/>
@@ -15697,7 +15540,7 @@
         <v>25</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>716</v>
+        <v>709</v>
       </c>
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>
@@ -15712,7 +15555,7 @@
         <v>17</v>
       </c>
       <c r="C2" s="18" t="s">
-        <v>719</v>
+        <v>712</v>
       </c>
       <c r="D2" s="3"/>
       <c r="E2" s="3"/>
@@ -15768,7 +15611,7 @@
         <v>25</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>716</v>
+        <v>709</v>
       </c>
       <c r="D6" s="3"/>
       <c r="E6" s="3"/>
@@ -15906,766 +15749,403 @@
 
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A154B75B-3F35-4B39-8504-480126E6D449}">
-  <dimension ref="A1:N20"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr defaultRowHeight="14.6"/>
   <cols>
-    <col min="1" max="1" width="18.23046875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="41.84375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="37.53515625" customWidth="1"/>
-    <col min="3" max="3" width="16.23046875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="74.53515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="21.3828125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.3046875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="21.4609375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="71.15234375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="15.45">
-      <c r="A1" s="15" t="s">
-        <v>4</v>
-      </c>
-      <c r="B1" s="6" t="s">
-        <v>683</v>
-      </c>
-      <c r="C1" s="3"/>
+    <row r="1" spans="1:7" ht="15.45">
+      <c r="A1" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>709</v>
+      </c>
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>
       <c r="F1" s="3"/>
       <c r="G1" s="3"/>
-      <c r="H1" s="3"/>
-      <c r="I1" s="3"/>
-      <c r="J1" s="3"/>
-      <c r="K1" s="3"/>
-      <c r="L1" s="3"/>
-      <c r="M1" s="3"/>
-      <c r="N1" s="3"/>
-    </row>
-    <row r="2" spans="1:14" ht="15.45">
-      <c r="A2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>684</v>
-      </c>
-      <c r="C2" s="3"/>
+    </row>
+    <row r="2" spans="1:7" ht="15.45">
+      <c r="A2" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C2" s="18" t="s">
+        <v>713</v>
+      </c>
       <c r="D2" s="3"/>
       <c r="E2" s="3"/>
       <c r="F2" s="3"/>
       <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
-      <c r="I2" s="3"/>
-      <c r="J2" s="3"/>
-      <c r="K2" s="3"/>
-      <c r="L2" s="3"/>
-      <c r="M2" s="3"/>
-      <c r="N2" s="3"/>
-    </row>
-    <row r="3" spans="1:14" ht="15.45">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
+    </row>
+    <row r="3" spans="1:7" ht="15.45">
+      <c r="A3" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" s="18" t="s">
+        <v>716</v>
+      </c>
       <c r="D3" s="3"/>
       <c r="E3" s="3"/>
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>
-      <c r="H3" s="3"/>
-      <c r="I3" s="3"/>
-      <c r="J3" s="3"/>
-      <c r="K3" s="3"/>
-      <c r="L3" s="3"/>
-      <c r="M3" s="3"/>
-      <c r="N3" s="3"/>
-    </row>
-    <row r="4" spans="1:14" ht="15.45">
-      <c r="A4" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="H4" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="I4" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="J4" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="K4" s="3"/>
-      <c r="L4" s="3"/>
-      <c r="M4" s="3"/>
-      <c r="N4" s="3"/>
-    </row>
-    <row r="5" spans="1:14" ht="15.45">
-      <c r="A5" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="C5" s="5"/>
-      <c r="D5" s="18" t="s">
-        <v>720</v>
-      </c>
-      <c r="E5" s="14"/>
-      <c r="F5" s="14"/>
-      <c r="G5" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="I5" s="3"/>
-      <c r="J5" s="3"/>
-      <c r="K5" s="3"/>
-      <c r="L5" s="3"/>
-      <c r="M5" s="3"/>
-      <c r="N5" s="3"/>
-    </row>
-    <row r="6" spans="1:14" ht="15.45">
-      <c r="A6" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="C6" s="5"/>
-      <c r="D6" s="18" t="s">
+    </row>
+    <row r="4" spans="1:7" ht="15.45">
+      <c r="A4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="18" t="s">
+        <v>683</v>
+      </c>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+    </row>
+    <row r="5" spans="1:7" ht="15.45">
+      <c r="A5" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>709</v>
+      </c>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+    </row>
+    <row r="6" spans="1:7" ht="15.45">
+      <c r="A6" s="9" t="s">
+        <v>532</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>444</v>
+      </c>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
+    </row>
+    <row r="7" spans="1:7" ht="15.45">
+      <c r="A7" s="9" t="s">
+        <v>684</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>683</v>
+      </c>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+    </row>
+    <row r="8" spans="1:7" ht="15.45">
+      <c r="A8" s="10" t="s">
         <v>685</v>
       </c>
-      <c r="E6" s="14"/>
-      <c r="F6" s="14"/>
-      <c r="G6" s="3"/>
-      <c r="H6" s="3"/>
-      <c r="I6" s="3"/>
-      <c r="J6" s="3"/>
-      <c r="K6" s="3"/>
-      <c r="L6" s="3"/>
-      <c r="M6" s="3"/>
-      <c r="N6" s="3"/>
-    </row>
-    <row r="7" spans="1:14" ht="15.45">
-      <c r="A7" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="B7" s="5"/>
-      <c r="C7" s="5"/>
-      <c r="D7" s="18" t="s">
-        <v>686</v>
-      </c>
-      <c r="E7" s="14"/>
-      <c r="F7" s="14"/>
-      <c r="G7" s="3"/>
-      <c r="H7" s="3"/>
-      <c r="I7" s="3"/>
-      <c r="J7" s="3"/>
-      <c r="K7" s="3"/>
-      <c r="L7" s="3"/>
-      <c r="M7" s="3"/>
-      <c r="N7" s="3"/>
-    </row>
-    <row r="8" spans="1:14" ht="15.45">
-      <c r="A8" s="3"/>
-      <c r="B8" s="3"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="17"/>
+      <c r="B8" s="10"/>
+      <c r="C8" s="10"/>
+      <c r="D8" s="3"/>
       <c r="E8" s="3"/>
       <c r="F8" s="3"/>
       <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
-      <c r="I8" s="3"/>
-      <c r="J8" s="3"/>
-      <c r="K8" s="3"/>
-      <c r="L8" s="3"/>
-      <c r="M8" s="3"/>
-      <c r="N8" s="3"/>
-    </row>
-    <row r="9" spans="1:14" ht="15.45">
-      <c r="A9" s="3"/>
-      <c r="B9" s="15"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
-      <c r="F9" s="3"/>
-      <c r="G9" s="3"/>
-      <c r="H9" s="3"/>
-      <c r="I9" s="3"/>
-      <c r="J9" s="3"/>
-      <c r="K9" s="3"/>
-      <c r="L9" s="3"/>
-      <c r="M9" s="3"/>
-      <c r="N9" s="3"/>
-    </row>
-    <row r="10" spans="1:14" ht="15.45">
-      <c r="A10" s="1"/>
-      <c r="B10" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="C10" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="D10" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="E10" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="F10" s="13" t="s">
-        <v>12</v>
-      </c>
-      <c r="G10" s="1"/>
-      <c r="H10" s="1"/>
-      <c r="I10" s="3"/>
-      <c r="J10" s="3"/>
-      <c r="K10" s="3"/>
-      <c r="L10" s="3"/>
-      <c r="M10" s="3"/>
-      <c r="N10" s="3"/>
-    </row>
-    <row r="11" spans="1:14" ht="15.45">
-      <c r="A11" s="3"/>
-      <c r="B11" s="9" t="s">
+    </row>
+    <row r="9" spans="1:7">
+      <c r="A9" s="20" t="s">
+        <v>686</v>
+      </c>
+      <c r="B9" s="20" t="s">
         <v>687</v>
       </c>
-      <c r="C11" s="10" t="s">
-        <v>54</v>
-      </c>
-      <c r="D11" s="11" t="s">
-        <v>444</v>
-      </c>
-      <c r="E11" s="10"/>
-      <c r="F11" s="10"/>
-      <c r="G11" s="3"/>
-      <c r="H11" s="3"/>
-      <c r="I11" s="3"/>
-      <c r="J11" s="3"/>
-      <c r="K11" s="3"/>
-      <c r="L11" s="3"/>
-      <c r="M11" s="3"/>
-      <c r="N11" s="3"/>
-    </row>
-    <row r="12" spans="1:14" ht="15.45">
-      <c r="A12" s="3"/>
-      <c r="B12" s="9" t="s">
+      <c r="C9" s="20" t="s">
         <v>688</v>
       </c>
-      <c r="C12" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="D12" s="11" t="s">
-        <v>686</v>
-      </c>
-      <c r="E12" s="10"/>
-      <c r="F12" s="10"/>
-      <c r="G12" s="3"/>
-      <c r="H12" s="3"/>
-      <c r="I12" s="3"/>
-      <c r="J12" s="3"/>
-      <c r="K12" s="3"/>
-      <c r="L12" s="3"/>
-      <c r="M12" s="3"/>
-      <c r="N12" s="3"/>
-    </row>
-    <row r="13" spans="1:14" ht="15.45">
-      <c r="A13" s="3"/>
-      <c r="B13" s="10" t="s">
+    </row>
+    <row r="10" spans="1:7">
+      <c r="A10" s="20" t="s">
         <v>689</v>
       </c>
-      <c r="C13" s="10"/>
-      <c r="D13" s="10"/>
-      <c r="E13" s="10"/>
-      <c r="F13" s="10"/>
-      <c r="G13" s="3"/>
-      <c r="H13" s="3"/>
-      <c r="I13" s="3"/>
-      <c r="J13" s="3"/>
-      <c r="K13" s="3"/>
-      <c r="L13" s="3"/>
-      <c r="M13" s="3"/>
-      <c r="N13" s="3"/>
-    </row>
-    <row r="14" spans="1:14">
+      <c r="B10" s="20" t="s">
+        <v>269</v>
+      </c>
+      <c r="C10" s="20" t="s">
+        <v>690</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
+      <c r="A11" s="20" t="s">
+        <v>691</v>
+      </c>
+      <c r="B11" s="20" t="s">
+        <v>687</v>
+      </c>
+      <c r="C11" s="20" t="s">
+        <v>692</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="A12" s="20" t="s">
+        <v>693</v>
+      </c>
+      <c r="B12" s="20" t="s">
+        <v>269</v>
+      </c>
+      <c r="C12" s="20" t="s">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
+      <c r="A13" s="20" t="s">
+        <v>80</v>
+      </c>
+      <c r="B13" s="20" t="s">
+        <v>81</v>
+      </c>
+      <c r="C13" s="20" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7">
+      <c r="A14" s="20" t="s">
+        <v>695</v>
+      </c>
       <c r="B14" s="20" t="s">
-        <v>690</v>
+        <v>176</v>
       </c>
       <c r="C14" s="20" t="s">
-        <v>691</v>
-      </c>
-      <c r="D14" s="20" t="s">
-        <v>692</v>
-      </c>
-      <c r="E14" s="20"/>
-      <c r="F14" s="20"/>
-    </row>
-    <row r="15" spans="1:14">
+        <v>683</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7">
+      <c r="A15" s="20"/>
       <c r="B15" s="20" t="s">
-        <v>693</v>
+        <v>687</v>
       </c>
       <c r="C15" s="20" t="s">
-        <v>269</v>
-      </c>
-      <c r="D15" s="20" t="s">
-        <v>694</v>
-      </c>
-      <c r="E15" s="20"/>
-      <c r="F15" s="20"/>
-    </row>
-    <row r="16" spans="1:14">
-      <c r="B16" s="20" t="s">
-        <v>695</v>
-      </c>
-      <c r="C16" s="20" t="s">
-        <v>691</v>
-      </c>
-      <c r="D16" s="20" t="s">
         <v>696</v>
       </c>
-      <c r="E16" s="20"/>
-      <c r="F16" s="20"/>
-    </row>
-    <row r="17" spans="2:6">
-      <c r="B17" s="20" t="s">
-        <v>697</v>
-      </c>
-      <c r="C17" s="20" t="s">
-        <v>269</v>
-      </c>
-      <c r="D17" s="20" t="s">
-        <v>698</v>
-      </c>
-      <c r="E17" s="20"/>
-      <c r="F17" s="20"/>
-    </row>
-    <row r="18" spans="2:6">
-      <c r="B18" s="20" t="s">
-        <v>80</v>
-      </c>
-      <c r="C18" s="20" t="s">
-        <v>81</v>
-      </c>
-      <c r="D18" s="20" t="s">
-        <v>82</v>
-      </c>
-      <c r="E18" s="20"/>
-      <c r="F18" s="20"/>
-    </row>
-    <row r="19" spans="2:6">
-      <c r="B19" s="20" t="s">
-        <v>699</v>
-      </c>
-      <c r="C19" s="20" t="s">
-        <v>176</v>
-      </c>
-      <c r="D19" s="20" t="s">
-        <v>686</v>
-      </c>
-      <c r="E19" s="20"/>
-      <c r="F19" s="20"/>
-    </row>
-    <row r="20" spans="2:6">
-      <c r="B20" s="20"/>
-      <c r="C20" s="20" t="s">
-        <v>691</v>
-      </c>
-      <c r="D20" s="20" t="s">
-        <v>700</v>
-      </c>
-      <c r="E20" s="20"/>
-      <c r="F20" s="20"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A31BDA5B-9A4A-4068-B396-81A2CC12D43A}">
-  <dimension ref="A1:N20"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr defaultRowHeight="14.6"/>
   <cols>
-    <col min="1" max="1" width="18.23046875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="46.921875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="37.53515625" customWidth="1"/>
-    <col min="3" max="3" width="16.23046875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="74.53515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="21.3828125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.3046875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="21.4609375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="56.15234375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="15.45">
-      <c r="A1" s="15" t="s">
-        <v>4</v>
-      </c>
-      <c r="B1" s="6" t="s">
-        <v>701</v>
-      </c>
-      <c r="C1" s="3"/>
+    <row r="1" spans="1:7" ht="15.45">
+      <c r="A1" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>709</v>
+      </c>
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>
       <c r="F1" s="3"/>
       <c r="G1" s="3"/>
-      <c r="H1" s="3"/>
-      <c r="I1" s="3"/>
-      <c r="J1" s="3"/>
-      <c r="K1" s="3"/>
-      <c r="L1" s="3"/>
-      <c r="M1" s="3"/>
-      <c r="N1" s="3"/>
-    </row>
-    <row r="2" spans="1:14" ht="15.45">
-      <c r="A2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>702</v>
-      </c>
-      <c r="C2" s="3"/>
+    </row>
+    <row r="2" spans="1:7" ht="15.45">
+      <c r="A2" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C2" s="18" t="s">
+        <v>714</v>
+      </c>
       <c r="D2" s="3"/>
       <c r="E2" s="3"/>
       <c r="F2" s="3"/>
       <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
-      <c r="I2" s="3"/>
-      <c r="J2" s="3"/>
-      <c r="K2" s="3"/>
-      <c r="L2" s="3"/>
-      <c r="M2" s="3"/>
-      <c r="N2" s="3"/>
-    </row>
-    <row r="3" spans="1:14" ht="15.45">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
+    </row>
+    <row r="3" spans="1:7" ht="15.45">
+      <c r="A3" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" s="18" t="s">
+        <v>715</v>
+      </c>
       <c r="D3" s="3"/>
       <c r="E3" s="3"/>
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>
-      <c r="H3" s="3"/>
-      <c r="I3" s="3"/>
-      <c r="J3" s="3"/>
-      <c r="K3" s="3"/>
-      <c r="L3" s="3"/>
-      <c r="M3" s="3"/>
-      <c r="N3" s="3"/>
-    </row>
-    <row r="4" spans="1:14" ht="15.45">
-      <c r="A4" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="H4" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="I4" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="J4" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="K4" s="3"/>
-      <c r="L4" s="3"/>
-      <c r="M4" s="3"/>
-      <c r="N4" s="3"/>
-    </row>
-    <row r="5" spans="1:14" ht="15.45">
-      <c r="A5" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="C5" s="5"/>
-      <c r="D5" s="18" t="s">
-        <v>721</v>
-      </c>
-      <c r="E5" s="14"/>
-      <c r="F5" s="14"/>
-      <c r="G5" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="I5" s="3"/>
-      <c r="J5" s="3"/>
-      <c r="K5" s="3"/>
-      <c r="L5" s="3"/>
-      <c r="M5" s="3"/>
-      <c r="N5" s="3"/>
-    </row>
-    <row r="6" spans="1:14" ht="15.45">
-      <c r="A6" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="C6" s="5"/>
-      <c r="D6" s="18" t="s">
-        <v>703</v>
-      </c>
-      <c r="E6" s="14"/>
-      <c r="F6" s="14"/>
+    </row>
+    <row r="4" spans="1:7" ht="15.45">
+      <c r="A4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="18" t="s">
+        <v>697</v>
+      </c>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+    </row>
+    <row r="5" spans="1:7" ht="15.45">
+      <c r="A5" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>709</v>
+      </c>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+    </row>
+    <row r="6" spans="1:7" ht="15.45">
+      <c r="A6" s="9" t="s">
+        <v>532</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>444</v>
+      </c>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
       <c r="G6" s="3"/>
-      <c r="H6" s="3"/>
-      <c r="I6" s="3"/>
-      <c r="J6" s="3"/>
-      <c r="K6" s="3"/>
-      <c r="L6" s="3"/>
-      <c r="M6" s="3"/>
-      <c r="N6" s="3"/>
-    </row>
-    <row r="7" spans="1:14" ht="15.45">
-      <c r="A7" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="B7" s="5"/>
-      <c r="C7" s="5"/>
-      <c r="D7" s="18" t="s">
-        <v>704</v>
-      </c>
-      <c r="E7" s="14"/>
-      <c r="F7" s="14"/>
+    </row>
+    <row r="7" spans="1:7" ht="15.45">
+      <c r="A7" s="9" t="s">
+        <v>698</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>697</v>
+      </c>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
       <c r="G7" s="3"/>
-      <c r="H7" s="3"/>
-      <c r="I7" s="3"/>
-      <c r="J7" s="3"/>
-      <c r="K7" s="3"/>
-      <c r="L7" s="3"/>
-      <c r="M7" s="3"/>
-      <c r="N7" s="3"/>
-    </row>
-    <row r="8" spans="1:14" ht="15.45">
-      <c r="A8" s="3"/>
-      <c r="B8" s="3"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="17"/>
+    </row>
+    <row r="8" spans="1:7" ht="15.45">
+      <c r="A8" s="10" t="s">
+        <v>699</v>
+      </c>
+      <c r="B8" s="10"/>
+      <c r="C8" s="10"/>
+      <c r="D8" s="3"/>
       <c r="E8" s="3"/>
       <c r="F8" s="3"/>
       <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
-      <c r="I8" s="3"/>
-      <c r="J8" s="3"/>
-      <c r="K8" s="3"/>
-      <c r="L8" s="3"/>
-      <c r="M8" s="3"/>
-      <c r="N8" s="3"/>
-    </row>
-    <row r="9" spans="1:14" ht="15.45">
-      <c r="A9" s="3"/>
-      <c r="B9" s="15"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
-      <c r="F9" s="3"/>
-      <c r="G9" s="3"/>
-      <c r="H9" s="3"/>
-      <c r="I9" s="3"/>
-      <c r="J9" s="3"/>
-      <c r="K9" s="3"/>
-      <c r="L9" s="3"/>
-      <c r="M9" s="3"/>
-      <c r="N9" s="3"/>
-    </row>
-    <row r="10" spans="1:14" ht="15.45">
-      <c r="A10" s="1"/>
-      <c r="B10" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="C10" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="D10" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="E10" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="F10" s="13" t="s">
-        <v>12</v>
-      </c>
-      <c r="G10" s="1"/>
-      <c r="H10" s="1"/>
-      <c r="I10" s="3"/>
-      <c r="J10" s="3"/>
-      <c r="K10" s="3"/>
-      <c r="L10" s="3"/>
-      <c r="M10" s="3"/>
-      <c r="N10" s="3"/>
-    </row>
-    <row r="11" spans="1:14" ht="15.45">
-      <c r="A11" s="3"/>
-      <c r="C11" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="D11" s="10" t="s">
-        <v>444</v>
-      </c>
-      <c r="E11" s="10"/>
-      <c r="F11" s="10"/>
-      <c r="G11" s="3"/>
-      <c r="H11" s="3"/>
-      <c r="I11" s="3"/>
-      <c r="J11" s="3"/>
-      <c r="K11" s="3"/>
-      <c r="L11" s="3"/>
-      <c r="M11" s="3"/>
-      <c r="N11" s="3"/>
-    </row>
-    <row r="12" spans="1:14" ht="15.45">
-      <c r="A12" s="3"/>
-      <c r="B12" s="9" t="s">
+    </row>
+    <row r="9" spans="1:7">
+      <c r="A9" s="20" t="s">
+        <v>700</v>
+      </c>
+      <c r="B9" s="20" t="s">
+        <v>75</v>
+      </c>
+      <c r="C9" s="20" t="s">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
+      <c r="A10" s="20"/>
+      <c r="B10" s="20" t="s">
+        <v>590</v>
+      </c>
+      <c r="C10" s="20"/>
+    </row>
+    <row r="11" spans="1:7">
+      <c r="A11" s="20" t="s">
+        <v>80</v>
+      </c>
+      <c r="B11" s="20" t="s">
+        <v>81</v>
+      </c>
+      <c r="C11" s="20" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="A12" s="20" t="s">
+        <v>701</v>
+      </c>
+      <c r="B12" s="20"/>
+      <c r="C12" s="20" t="s">
+        <v>702</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
+      <c r="A13" s="20" t="s">
+        <v>703</v>
+      </c>
+      <c r="B13" s="20"/>
+      <c r="C13" s="20" t="s">
+        <v>704</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7">
+      <c r="A14" s="20" t="s">
         <v>705</v>
       </c>
-      <c r="C12" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="D12" s="11" t="s">
-        <v>704</v>
-      </c>
-      <c r="E12" s="10"/>
-      <c r="F12" s="10"/>
-      <c r="G12" s="3"/>
-      <c r="H12" s="3"/>
-      <c r="I12" s="3"/>
-      <c r="J12" s="3"/>
-      <c r="K12" s="3"/>
-      <c r="L12" s="3"/>
-      <c r="M12" s="3"/>
-      <c r="N12" s="3"/>
-    </row>
-    <row r="13" spans="1:14" ht="15.45">
-      <c r="A13" s="3"/>
-      <c r="B13" s="10" t="s">
+      <c r="B14" s="20"/>
+      <c r="C14" s="20" t="s">
         <v>706</v>
       </c>
-      <c r="C13" s="10"/>
-      <c r="D13" s="10"/>
-      <c r="E13" s="10"/>
-      <c r="F13" s="10"/>
-      <c r="G13" s="3"/>
-      <c r="H13" s="3"/>
-      <c r="I13" s="3"/>
-      <c r="J13" s="3"/>
-      <c r="K13" s="3"/>
-      <c r="L13" s="3"/>
-      <c r="M13" s="3"/>
-      <c r="N13" s="3"/>
-    </row>
-    <row r="14" spans="1:14">
-      <c r="B14" s="20" t="s">
+    </row>
+    <row r="15" spans="1:7">
+      <c r="A15" s="20" t="s">
         <v>707</v>
       </c>
-      <c r="C14" s="20" t="s">
-        <v>75</v>
-      </c>
-      <c r="D14" s="20" t="s">
-        <v>698</v>
-      </c>
-      <c r="E14" s="20"/>
-      <c r="F14" s="20"/>
-    </row>
-    <row r="15" spans="1:14">
       <c r="B15" s="20"/>
       <c r="C15" s="20" t="s">
-        <v>590</v>
-      </c>
-      <c r="D15" s="20"/>
-      <c r="E15" s="20"/>
-      <c r="F15" s="20"/>
-    </row>
-    <row r="16" spans="1:14">
-      <c r="B16" s="20" t="s">
-        <v>80</v>
-      </c>
-      <c r="C16" s="20" t="s">
-        <v>81</v>
-      </c>
-      <c r="D16" s="20" t="s">
-        <v>82</v>
-      </c>
-      <c r="E16" s="20"/>
-      <c r="F16" s="20"/>
-    </row>
-    <row r="17" spans="2:6">
-      <c r="B17" s="20" t="s">
         <v>708</v>
       </c>
-      <c r="C17" s="20"/>
-      <c r="D17" s="20" t="s">
-        <v>709</v>
-      </c>
-      <c r="E17" s="20"/>
-      <c r="F17" s="20"/>
-    </row>
-    <row r="18" spans="2:6">
-      <c r="B18" s="20" t="s">
-        <v>710</v>
-      </c>
-      <c r="C18" s="20"/>
-      <c r="D18" s="20" t="s">
-        <v>711</v>
-      </c>
-      <c r="E18" s="20"/>
-      <c r="F18" s="20"/>
-    </row>
-    <row r="19" spans="2:6">
-      <c r="B19" s="20" t="s">
-        <v>712</v>
-      </c>
-      <c r="C19" s="20"/>
-      <c r="D19" s="20" t="s">
-        <v>713</v>
-      </c>
-      <c r="E19" s="20"/>
-      <c r="F19" s="20"/>
-    </row>
-    <row r="20" spans="2:6">
-      <c r="B20" s="20" t="s">
-        <v>714</v>
-      </c>
-      <c r="C20" s="20"/>
-      <c r="D20" s="20" t="s">
-        <v>715</v>
-      </c>
-      <c r="E20" s="20"/>
-      <c r="F20" s="20"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>